<commit_message>
Parece ir bien los eventos pero falla lel cruce y mutacion
</commit_message>
<xml_diff>
--- a/db/Profesor.xlsx
+++ b/db/Profesor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PosGrado\Proyecto Titulacion\Timetabling\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FAC80DA-00FA-4080-A185-539745E43428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FF0F6FD-0038-4BDB-A979-814F3A1DD9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3975" yWindow="4695" windowWidth="28785" windowHeight="15345" xr2:uid="{5C1DD6D8-1001-4079-A3F5-95F5066F8827}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{5C1DD6D8-1001-4079-A3F5-95F5066F8827}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -192,9 +192,6 @@
     <t>Item</t>
   </si>
   <si>
-    <t>Dirección</t>
-  </si>
-  <si>
     <t>Guitarra</t>
   </si>
   <si>
@@ -217,6 +214,9 @@
   </si>
   <si>
     <t>Percusion</t>
+  </si>
+  <si>
+    <t>Direccion</t>
   </si>
 </sst>
 </file>
@@ -585,7 +585,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -602,7 +602,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
         <v>51</v>
@@ -619,7 +619,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
         <v>51</v>
@@ -636,7 +636,7 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
         <v>51</v>
@@ -653,7 +653,7 @@
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
         <v>51</v>
@@ -670,7 +670,7 @@
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s">
         <v>51</v>
@@ -687,7 +687,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
         <v>51</v>
@@ -704,7 +704,7 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
         <v>51</v>
@@ -721,7 +721,7 @@
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E9" t="s">
         <v>51</v>
@@ -738,7 +738,7 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E10" t="s">
         <v>51</v>
@@ -755,7 +755,7 @@
         <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
         <v>51</v>
@@ -772,7 +772,7 @@
         <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E12" t="s">
         <v>51</v>
@@ -786,10 +786,10 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E13" t="s">
         <v>51</v>
@@ -806,7 +806,7 @@
         <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E14" t="s">
         <v>51</v>
@@ -823,7 +823,7 @@
         <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E15" t="s">
         <v>51</v>
@@ -840,7 +840,7 @@
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E16" t="s">
         <v>51</v>
@@ -857,7 +857,7 @@
         <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E17" t="s">
         <v>51</v>
@@ -874,7 +874,7 @@
         <v>5</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
         <v>51</v>
@@ -891,7 +891,7 @@
         <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
         <v>50</v>
@@ -908,7 +908,7 @@
         <v>31</v>
       </c>
       <c r="D20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E20" t="s">
         <v>50</v>
@@ -925,7 +925,7 @@
         <v>33</v>
       </c>
       <c r="D21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E21" t="s">
         <v>50</v>
@@ -942,7 +942,7 @@
         <v>29</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E22" t="s">
         <v>50</v>
@@ -959,7 +959,7 @@
         <v>38</v>
       </c>
       <c r="D23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E23" t="s">
         <v>50</v>
@@ -976,7 +976,7 @@
         <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E24" t="s">
         <v>50</v>
@@ -993,7 +993,7 @@
         <v>40</v>
       </c>
       <c r="D25" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E25" t="s">
         <v>50</v>
@@ -1010,7 +1010,7 @@
         <v>46</v>
       </c>
       <c r="D26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E26" t="s">
         <v>50</v>
@@ -1027,7 +1027,7 @@
         <v>48</v>
       </c>
       <c r="D27" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E27" t="s">
         <v>50</v>

</xml_diff>